<commit_message>
Release 0.1.1: comment-bound named parameters with real sample values (valid-Excel templates)
</commit_message>
<xml_diff>
--- a/templates/sales_receipt_template.xlsx
+++ b/templates/sales_receipt_template.xlsx
@@ -13,42 +13,107 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0">
+      <text>
+        <t>#receipt</t>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0">
+      <text>
+        <t>#date</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t>#customer</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0">
+      <text>
+        <t>#address</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0">
+      <text>
+        <t>#qty</t>
+      </text>
+    </comment>
+    <comment ref="C7" authorId="0">
+      <text>
+        <t>#desc</t>
+      </text>
+    </comment>
+    <comment ref="D7" authorId="0">
+      <text>
+        <t>#price</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0">
+      <text>
+        <t>#qty</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0">
+      <text>
+        <t>#desc</t>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0">
+      <text>
+        <t>#price</t>
+      </text>
+    </comment>
+    <comment ref="D11" authorId="0">
+      <text>
+        <t>#taxrate</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>SALES RECEIPT</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>header(date,receipt,customer,address)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Receipt #:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Date:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1/5/2009</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>header</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Receipt #:</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>${2}</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Date:</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>${1}</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Sold To:</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>${3}</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>${4}</t>
+    <t>Jose Maria Fernandez</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1010 Broadway, New York, NY 10010</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -68,19 +133,31 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>row1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>row2</t>
+    <t>row1(seq,qty,desc,price)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Introduction to Algebra</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>row2(seq,qty,desc,price)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Introduction to Algebra Solutions Manual</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>footer(taxrate)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Subtotal:</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>footer</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Subtotal:</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -473,19 +550,19 @@
       <c r="B2" t="s" s="3">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>22215</v>
+      </c>
+      <c r="D2" t="s" s="4">
         <v>3</v>
       </c>
-      <c r="D2" t="s" s="4">
+      <c r="E2" t="s" s="5">
         <v>4</v>
-      </c>
-      <c r="E2" t="s" s="5">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s" s="3">
         <v>6</v>
@@ -496,7 +573,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
@@ -520,14 +597,14 @@
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s" s="5">
-        <v>3</v>
+      <c r="B7" s="5">
+        <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s" s="8">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="D7" s="8">
+        <v>53</v>
       </c>
       <c r="E7" s="8">
         <f>B7*D7</f>
@@ -536,16 +613,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="9">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s" s="10">
+        <v>16</v>
+      </c>
+      <c r="D8" s="11">
         <v>14</v>
-      </c>
-      <c r="B8" t="s" s="9">
-        <v>3</v>
-      </c>
-      <c r="C8" t="s" s="10">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s" s="11">
-        <v>8</v>
       </c>
       <c r="E8" s="11">
         <f>B8*D8</f>
@@ -554,25 +631,25 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s" s="4">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E10" s="8">
-        <f>SUM(E${firstrow}:E${lastrow})</f>
+        <f>SUM(E$7:E8)</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s" s="12">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0.0525</v>
       </c>
       <c r="E11" s="8">
         <f>E10*D11</f>
@@ -581,10 +658,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E12" s="13">
         <f>E10+E11</f>
@@ -599,5 +676,6 @@
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Release 0.2.0: Excel-template workflow only; remove declarative engine; PDF via optional LibreOffice (pdf feature); README design guide + screenshots
</commit_message>
<xml_diff>
--- a/templates/sales_receipt_template.xlsx
+++ b/templates/sales_receipt_template.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>SALES RECEIPT</t>
     <phoneticPr fontId="1"/>
@@ -93,11 +93,15 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>NNNNN</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>Date:</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>1/5/2009</t>
+    <t>MM/DD/YYYY</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -109,11 +113,11 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Jose Maria Fernandez</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>1010 Broadway, New York, NY 10010</t>
+    <t>Customer Name</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Street, City, State ZIP</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -137,7 +141,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Introduction to Algebra</t>
+    <t>Sample item</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -145,7 +149,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Introduction to Algebra Solutions Manual</t>
+    <t>Another sample item</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -532,7 +536,7 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
     <col min="4" max="5" width="13" customWidth="1"/>
@@ -550,61 +554,61 @@
       <c r="B2" t="s" s="3">
         <v>2</v>
       </c>
-      <c r="C2">
-        <v>22215</v>
+      <c r="C2" t="s">
+        <v>3</v>
       </c>
       <c r="D2" t="s" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="s" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s" s="6">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s" s="6">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="8">
-        <v>53</v>
+        <v>9.99</v>
       </c>
       <c r="E7" s="8">
         <f>B7*D7</f>
@@ -613,16 +617,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s" s="10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" s="11">
-        <v>14</v>
+        <v>4.99</v>
       </c>
       <c r="E8" s="11">
         <f>B8*D8</f>
@@ -631,10 +635,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10" s="8">
         <f>SUM(E$7:E8)</f>
@@ -643,13 +647,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D11" s="12">
-        <v>0.0525</v>
+        <v>0.1</v>
       </c>
       <c r="E11" s="8">
         <f>E10*D11</f>
@@ -658,10 +662,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" s="13">
         <f>E10+E11</f>

</xml_diff>